<commit_message>
Add Phase 8 statistical validation and update project files
</commit_message>
<xml_diff>
--- a/project_files/DA418_S1_Progress Tracker.xlsx
+++ b/project_files/DA418_S1_Progress Tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Anitha\NIIT\Capstone Project\capstone-project-retail-tech\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Anitha\NIIT\Capstone Project\capstone-project-retail-tech\project_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2756DDC5-5B78-48D2-B8BF-4A9F9C5EE0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A4ECBF6-B720-459B-8B1D-524EF12608C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{EE05F723-CC45-4365-ABE9-4CF4A7CBB336}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{EE05F723-CC45-4365-ABE9-4CF4A7CBB336}"/>
   </bookViews>
   <sheets>
     <sheet name="Phase 1" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="107">
   <si>
     <t>Capstone Project - Phase 1 End Tracker</t>
   </si>
@@ -391,6 +391,21 @@
   </si>
   <si>
     <t>Phase 7</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1x9iJTYemhv0lsci7wYLtiDzuj9jv52Mt/view?usp=sharing</t>
+  </si>
+  <si>
+    <t>Nil</t>
+  </si>
+  <si>
+    <t>E-Commerce Sales &amp; Customer Analysis</t>
+  </si>
+  <si>
+    <t>Phase 8</t>
+  </si>
+  <si>
+    <t>Phase 9</t>
   </si>
 </sst>
 </file>
@@ -659,7 +674,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -760,74 +775,80 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1758,13 +1779,13 @@
       <c r="B4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="49" t="s">
+      <c r="C4" s="47" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="51"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="49"/>
     </row>
     <row r="5" spans="2:8" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
@@ -1780,45 +1801,45 @@
       <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="39" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-      <c r="G6" s="45"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="52"/>
     </row>
     <row r="7" spans="2:8" ht="18" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="45"/>
+        <v>104</v>
+      </c>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="41"/>
     </row>
     <row r="8" spans="2:8" ht="18" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="52">
+      <c r="C8" s="50">
         <v>46252</v>
       </c>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="45"/>
+      <c r="D8" s="51"/>
+      <c r="E8" s="51"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="52"/>
     </row>
     <row r="9" spans="2:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="B9" s="46"/>
-      <c r="C9" s="47"/>
-      <c r="D9" s="47"/>
-      <c r="E9" s="47"/>
-      <c r="F9" s="47"/>
-      <c r="G9" s="48"/>
+      <c r="B9" s="44"/>
+      <c r="C9" s="45"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="46"/>
     </row>
     <row r="10" spans="2:8" s="1" customFormat="1" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
@@ -2081,37 +2102,37 @@
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="56"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="45"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="41"/>
     </row>
     <row r="4" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="56"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="45"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="41"/>
     </row>
     <row r="5" spans="2:9" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="56"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="45"/>
+      <c r="C5" s="62"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="41"/>
     </row>
     <row r="6" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="56"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="45"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="41"/>
     </row>
     <row r="7" spans="2:9" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:9" s="9" customFormat="1" ht="121.8" x14ac:dyDescent="0.3">
@@ -2328,56 +2349,56 @@
       <c r="C3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="45"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="41"/>
       <c r="H3" s="10"/>
     </row>
     <row r="4" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="56"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="45"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="41"/>
       <c r="H4" s="10"/>
     </row>
     <row r="5" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="56" t="s">
+      <c r="C5" s="62" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="45"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="41"/>
       <c r="H5" s="10"/>
     </row>
     <row r="6" spans="2:11" ht="36" x14ac:dyDescent="0.35">
       <c r="B6" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="56"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-      <c r="G6" s="45"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="41"/>
       <c r="H6" s="10"/>
     </row>
     <row r="7" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="52"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="45"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="41"/>
       <c r="H7" s="10"/>
     </row>
     <row r="9" spans="2:11" s="28" customFormat="1" ht="87" x14ac:dyDescent="0.3">
@@ -2695,13 +2716,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
     </row>
     <row r="2" spans="2:9" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="25" t="s">
@@ -2711,51 +2732,51 @@
         <v>2</v>
       </c>
       <c r="D2" s="25"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
     </row>
     <row r="3" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="58" t="s">
+      <c r="C3" s="57" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
       <c r="F3" s="27"/>
     </row>
     <row r="4" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="58" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="59"/>
-      <c r="E4" s="59"/>
+      <c r="C4" s="57" t="s">
+        <v>104</v>
+      </c>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
       <c r="F4" s="27"/>
     </row>
     <row r="5" spans="2:9" ht="31.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="61" t="s">
+      <c r="C5" s="60" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
       <c r="F5" s="27"/>
     </row>
     <row r="6" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="60">
+      <c r="C6" s="59">
         <v>46254</v>
       </c>
-      <c r="D6" s="59"/>
-      <c r="E6" s="59"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
       <c r="F6" s="27"/>
     </row>
     <row r="8" spans="2:9" ht="69.599999999999994" x14ac:dyDescent="0.3">
@@ -2981,22 +3002,22 @@
       <c r="C3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="45"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="41"/>
     </row>
     <row r="4" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="45"/>
+        <v>104</v>
+      </c>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="41"/>
     </row>
     <row r="5" spans="2:11" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
@@ -3005,22 +3026,22 @@
       <c r="C5" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="45"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="41"/>
     </row>
     <row r="6" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="52">
+      <c r="C6" s="42">
         <v>46255</v>
       </c>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-      <c r="G6" s="45"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="41"/>
     </row>
     <row r="8" spans="2:11" ht="87" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
@@ -3275,22 +3296,22 @@
       <c r="C3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="41"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="52"/>
     </row>
     <row r="4" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="41"/>
+        <v>104</v>
+      </c>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="52"/>
     </row>
     <row r="5" spans="2:11" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
@@ -3299,22 +3320,22 @@
       <c r="C5" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="45"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="41"/>
     </row>
     <row r="6" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="42">
+      <c r="C6" s="50">
         <v>46258</v>
       </c>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="41"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="52"/>
     </row>
     <row r="8" spans="2:11" ht="87" x14ac:dyDescent="0.3">
       <c r="B8" s="15" t="s">
@@ -3569,22 +3590,22 @@
       <c r="C3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="41"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="52"/>
     </row>
     <row r="4" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="41"/>
+        <v>104</v>
+      </c>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="52"/>
     </row>
     <row r="5" spans="2:11" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
@@ -3593,22 +3614,22 @@
       <c r="C5" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="45"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="41"/>
     </row>
     <row r="6" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="42">
+      <c r="C6" s="50">
         <v>46259</v>
       </c>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="41"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="52"/>
     </row>
     <row r="8" spans="2:11" ht="87" x14ac:dyDescent="0.3">
       <c r="B8" s="15" t="s">
@@ -3826,7 +3847,7 @@
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
     <col min="3" max="3" width="45.88671875" customWidth="1"/>
-    <col min="4" max="4" width="27" customWidth="1"/>
+    <col min="4" max="4" width="76.6640625" customWidth="1"/>
     <col min="5" max="5" width="18.5546875" customWidth="1"/>
     <col min="6" max="6" width="27.44140625" customWidth="1"/>
     <col min="7" max="7" width="18.6640625" customWidth="1"/>
@@ -3861,20 +3882,20 @@
       <c r="C3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
     </row>
     <row r="4" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
+        <v>104</v>
+      </c>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
     </row>
     <row r="5" spans="2:9" ht="38.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
@@ -3883,22 +3904,22 @@
       <c r="C5" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
     </row>
     <row r="6" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="52">
+      <c r="C6" s="42">
         <v>46261</v>
       </c>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-    </row>
-    <row r="8" spans="2:9" ht="54" x14ac:dyDescent="0.3">
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+    </row>
+    <row r="8" spans="2:9" ht="52.2" x14ac:dyDescent="0.3">
       <c r="B8" s="15" t="s">
         <v>9</v>
       </c>
@@ -3931,8 +3952,12 @@
       <c r="C9" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="D9" s="33" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>103</v>
+      </c>
       <c r="F9" s="18"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -4074,7 +4099,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B22">
         <v>1</v>
       </c>
@@ -4100,7 +4125,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B23">
         <v>2</v>
       </c>
@@ -4189,9 +4214,10 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C5" r:id="rId1" xr:uid="{48B31ECC-3FAC-42C6-B0FF-1E13E6B894E7}"/>
+    <hyperlink ref="D9" r:id="rId2" xr:uid="{6AFDE3F1-96CC-486B-A5B3-9244D49A5BAD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -4244,24 +4270,24 @@
       <c r="C3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="45"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="41"/>
     </row>
     <row r="4" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="44"/>
-      <c r="H4" s="45"/>
+        <v>104</v>
+      </c>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="41"/>
     </row>
     <row r="5" spans="2:11" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
@@ -4270,24 +4296,24 @@
       <c r="C5" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="45"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="41"/>
     </row>
     <row r="6" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="52">
+      <c r="C6" s="42">
         <v>46262</v>
       </c>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-      <c r="G6" s="44"/>
-      <c r="H6" s="45"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="41"/>
     </row>
     <row r="8" spans="2:11" s="1" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="B8" s="17" t="s">
@@ -4325,15 +4351,29 @@
       <c r="B9" s="5">
         <v>1</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="2"/>
+      <c r="C9" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="E9" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="F9" s="64" t="s">
+        <v>94</v>
+      </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="H9" s="64" t="s">
+        <v>75</v>
+      </c>
+      <c r="I9" s="32">
+        <v>46267</v>
+      </c>
       <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
+      <c r="K9" s="64" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="10" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B10" s="5">
@@ -4526,24 +4566,24 @@
       <c r="C3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="41"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="52"/>
     </row>
     <row r="4" spans="2:10" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="41"/>
+        <v>104</v>
+      </c>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="51"/>
+      <c r="H4" s="52"/>
     </row>
     <row r="5" spans="2:10" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
@@ -4552,24 +4592,24 @@
       <c r="C5" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="45"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="41"/>
     </row>
     <row r="6" spans="2:10" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="42">
-        <v>46265</v>
-      </c>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="41"/>
+      <c r="C6" s="50">
+        <v>46266</v>
+      </c>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="51"/>
+      <c r="H6" s="52"/>
     </row>
     <row r="8" spans="2:10" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="B8" s="15" t="s">
@@ -4604,14 +4644,26 @@
       <c r="B9" s="20">
         <v>1</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="C9" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="E9" s="63" t="s">
+        <v>94</v>
+      </c>
       <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
+      <c r="G9" s="64" t="s">
+        <v>75</v>
+      </c>
+      <c r="H9" s="32">
+        <v>46267</v>
+      </c>
       <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
+      <c r="J9" s="2" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="10" spans="2:10" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B10" s="5">
@@ -4793,24 +4845,24 @@
       <c r="C3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="41"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="52"/>
     </row>
     <row r="4" spans="2:10" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="41"/>
+        <v>104</v>
+      </c>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="51"/>
+      <c r="H4" s="52"/>
     </row>
     <row r="5" spans="2:10" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
@@ -4819,23 +4871,21 @@
       <c r="C5" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="45"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="41"/>
     </row>
     <row r="6" spans="2:10" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="42">
-        <v>46266</v>
-      </c>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="41"/>
+      <c r="C6" s="50"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="52"/>
     </row>
     <row r="8" spans="2:10" s="9" customFormat="1" ht="156.6" x14ac:dyDescent="0.3">
       <c r="B8" s="15" t="s">
@@ -5014,15 +5064,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="b18f8198-02fb-408b-a649-baf04150ea28">
@@ -5031,6 +5072,15 @@
     <TaxCatchAll xmlns="0f01b7b4-d4b6-47da-93c5-cffa90a406b9" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5283,20 +5333,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E88113A-166D-44CD-886E-1102874B4258}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E8D7F3F-2EC6-459C-B8E1-5F91591B843B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="b18f8198-02fb-408b-a649-baf04150ea28"/>
     <ds:schemaRef ds:uri="0f01b7b4-d4b6-47da-93c5-cffa90a406b9"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E88113A-166D-44CD-886E-1102874B4258}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update project report, model, tracker and presentation
</commit_message>
<xml_diff>
--- a/project_files/DA418_S1_Progress Tracker.xlsx
+++ b/project_files/DA418_S1_Progress Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Anitha\NIIT\Capstone Project\capstone-project-retail-tech\project_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D48EF238-3174-4F63-A723-033697A14716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CDFC127-86F6-49C7-8C41-A53AF8E96E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="10" xr2:uid="{EE05F723-CC45-4365-ABE9-4CF4A7CBB336}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="110">
   <si>
     <t>Capstone Project - Phase 1 End Tracker</t>
   </si>
@@ -772,6 +772,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -787,16 +788,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -805,7 +797,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -825,6 +820,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -853,13 +857,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1752,14 +1752,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="28.2" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="38"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="39"/>
     </row>
     <row r="2" spans="2:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -1770,32 +1770,32 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="2:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="54" t="s">
+      <c r="C3" s="56" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="56"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="58"/>
     </row>
     <row r="4" spans="2:8" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="51" t="s">
+      <c r="C4" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="53"/>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="52"/>
     </row>
     <row r="5" spans="2:8" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
@@ -1811,45 +1811,45 @@
       <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="47" t="s">
+      <c r="C6" s="42" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="42"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="55"/>
     </row>
     <row r="7" spans="2:8" ht="18" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="47" t="s">
+      <c r="C7" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="46"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="44"/>
     </row>
     <row r="8" spans="2:8" ht="18" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="41">
+      <c r="C8" s="53">
         <v>46252</v>
       </c>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="43"/>
+      <c r="D8" s="54"/>
+      <c r="E8" s="54"/>
+      <c r="F8" s="54"/>
+      <c r="G8" s="55"/>
     </row>
     <row r="9" spans="2:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="B9" s="48"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="50"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="49"/>
     </row>
     <row r="10" spans="2:8" s="1" customFormat="1" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
@@ -2089,13 +2089,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="38"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="2" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -2105,44 +2105,44 @@
         <v>2</v>
       </c>
       <c r="D2" s="2"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="41"/>
     </row>
     <row r="3" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="44"/>
     </row>
     <row r="4" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="64"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="44"/>
     </row>
     <row r="5" spans="2:9" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="64"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="44"/>
     </row>
     <row r="6" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="64"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="46"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="44"/>
     </row>
     <row r="7" spans="2:9" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:9" s="9" customFormat="1" ht="121.8" x14ac:dyDescent="0.3">
@@ -2337,14 +2337,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="38"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="39"/>
       <c r="H1" s="9"/>
     </row>
     <row r="2" spans="2:11" ht="54" x14ac:dyDescent="0.35">
@@ -2356,67 +2356,67 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
       <c r="H2" s="9"/>
     </row>
     <row r="3" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="46"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="44"/>
       <c r="H3" s="10"/>
     </row>
     <row r="4" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="64"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="44"/>
       <c r="H4" s="10"/>
     </row>
     <row r="5" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="64" t="s">
+      <c r="C5" s="46" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="44"/>
       <c r="H5" s="10"/>
     </row>
     <row r="6" spans="2:11" ht="36" x14ac:dyDescent="0.35">
       <c r="B6" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="64"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="46"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="44"/>
       <c r="H6" s="10"/>
     </row>
     <row r="7" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="63"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="46"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="44"/>
       <c r="H7" s="10"/>
     </row>
     <row r="9" spans="2:11" s="28" customFormat="1" ht="87" x14ac:dyDescent="0.3">
@@ -2455,17 +2455,23 @@
       <c r="B10" s="5">
         <v>1</v>
       </c>
-      <c r="C10" s="18"/>
+      <c r="C10" s="18" t="s">
+        <v>90</v>
+      </c>
       <c r="D10" s="18" t="s">
         <v>90</v>
       </c>
       <c r="E10" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="F10" s="18"/>
+      <c r="F10" s="18" t="s">
+        <v>90</v>
+      </c>
       <c r="G10" s="30"/>
       <c r="H10" s="29"/>
-      <c r="I10" s="2"/>
+      <c r="I10" s="29">
+        <v>46271</v>
+      </c>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
@@ -2738,13 +2744,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
     </row>
     <row r="2" spans="2:9" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="25" t="s">
@@ -2754,51 +2760,51 @@
         <v>2</v>
       </c>
       <c r="D2" s="25"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
     </row>
     <row r="3" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="58" t="s">
+      <c r="C3" s="60" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
       <c r="F3" s="27"/>
     </row>
     <row r="4" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="58" t="s">
+      <c r="C4" s="60" t="s">
         <v>104</v>
       </c>
-      <c r="D4" s="59"/>
-      <c r="E4" s="59"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
       <c r="F4" s="27"/>
     </row>
     <row r="5" spans="2:9" ht="31.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="61" t="s">
+      <c r="C5" s="63" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
+      <c r="D5" s="61"/>
+      <c r="E5" s="61"/>
       <c r="F5" s="27"/>
     </row>
     <row r="6" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="60">
+      <c r="C6" s="62">
         <v>46254</v>
       </c>
-      <c r="D6" s="59"/>
-      <c r="E6" s="59"/>
+      <c r="D6" s="61"/>
+      <c r="E6" s="61"/>
       <c r="F6" s="27"/>
     </row>
     <row r="8" spans="2:9" ht="69.599999999999994" x14ac:dyDescent="0.3">
@@ -2996,14 +3002,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="38"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="39"/>
     </row>
     <row r="2" spans="2:11" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -3014,56 +3020,56 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="46"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="44"/>
     </row>
     <row r="4" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="47" t="s">
+      <c r="C4" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="46"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="44"/>
     </row>
     <row r="5" spans="2:11" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="65" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="44"/>
     </row>
     <row r="6" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="63">
+      <c r="C6" s="45">
         <v>46255</v>
       </c>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="46"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="44"/>
     </row>
     <row r="8" spans="2:11" ht="87" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
@@ -3290,14 +3296,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="38"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="39"/>
     </row>
     <row r="2" spans="2:11" ht="36" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -3308,56 +3314,56 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="43"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="55"/>
     </row>
     <row r="4" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="47" t="s">
+      <c r="C4" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="43"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="55"/>
     </row>
     <row r="5" spans="2:11" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="65" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="44"/>
     </row>
     <row r="6" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="41">
+      <c r="C6" s="53">
         <v>46258</v>
       </c>
-      <c r="D6" s="42"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="55"/>
     </row>
     <row r="8" spans="2:11" ht="87" x14ac:dyDescent="0.3">
       <c r="B8" s="15" t="s">
@@ -3584,14 +3590,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="38"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="39"/>
     </row>
     <row r="2" spans="2:11" ht="54" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -3602,56 +3608,56 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="43"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="55"/>
     </row>
     <row r="4" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="47" t="s">
+      <c r="C4" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="43"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="55"/>
     </row>
     <row r="5" spans="2:11" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="65" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="44"/>
     </row>
     <row r="6" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="41">
+      <c r="C6" s="53">
         <v>46259</v>
       </c>
-      <c r="D6" s="42"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="55"/>
     </row>
     <row r="8" spans="2:11" ht="87" x14ac:dyDescent="0.3">
       <c r="B8" s="15" t="s">
@@ -3878,13 +3884,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
     </row>
     <row r="2" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -3895,51 +3901,51 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="39"/>
+      <c r="F2" s="40"/>
     </row>
     <row r="3" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
     </row>
     <row r="4" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="47" t="s">
+      <c r="C4" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
     </row>
     <row r="5" spans="2:9" ht="38.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="65" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
     </row>
     <row r="6" spans="2:9" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="63">
+      <c r="C6" s="45">
         <v>46261</v>
       </c>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
     </row>
     <row r="8" spans="2:9" ht="52.2" x14ac:dyDescent="0.3">
       <c r="B8" s="15" t="s">
@@ -4262,15 +4268,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="38"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="39"/>
     </row>
     <row r="2" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -4282,60 +4288,60 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="46"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="47" t="s">
+      <c r="C4" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="46"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="44"/>
     </row>
     <row r="5" spans="2:11" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="65" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="46"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="2:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="63">
+      <c r="C6" s="45">
         <v>46262</v>
       </c>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
-      <c r="H6" s="46"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="44"/>
     </row>
     <row r="8" spans="2:11" s="1" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="B8" s="17" t="s">
@@ -4558,15 +4564,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="37" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="38"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="39"/>
     </row>
     <row r="2" spans="2:10" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -4578,60 +4584,60 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="2:10" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="43"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="55"/>
     </row>
     <row r="4" spans="2:10" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="47" t="s">
+      <c r="C4" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="43"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="55"/>
     </row>
     <row r="5" spans="2:10" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="65" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="46"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="2:10" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="41">
+      <c r="C6" s="53">
         <v>46266</v>
       </c>
-      <c r="D6" s="42"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="55"/>
     </row>
     <row r="8" spans="2:10" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="B8" s="15" t="s">
@@ -4839,14 +4845,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="38"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="39"/>
     </row>
     <row r="2" spans="2:10" ht="36" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -4857,57 +4863,57 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="2:10" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="43"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="55"/>
     </row>
     <row r="4" spans="2:10" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="47" t="s">
+      <c r="C4" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="43"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="55"/>
     </row>
     <row r="5" spans="2:10" ht="36" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="65" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="46"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="2:10" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="41"/>
-      <c r="D6" s="42"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="55"/>
     </row>
     <row r="8" spans="2:10" s="9" customFormat="1" ht="156.6" x14ac:dyDescent="0.3">
       <c r="B8" s="15" t="s">
@@ -4955,7 +4961,7 @@
       <c r="G9" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="65">
+      <c r="H9" s="36">
         <v>46270</v>
       </c>
       <c r="I9" s="18"/>
@@ -5098,15 +5104,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="b18f8198-02fb-408b-a649-baf04150ea28">
@@ -5115,6 +5112,15 @@
     <TaxCatchAll xmlns="0f01b7b4-d4b6-47da-93c5-cffa90a406b9" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5367,20 +5373,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E88113A-166D-44CD-886E-1102874B4258}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E8D7F3F-2EC6-459C-B8E1-5F91591B843B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="b18f8198-02fb-408b-a649-baf04150ea28"/>
     <ds:schemaRef ds:uri="0f01b7b4-d4b6-47da-93c5-cffa90a406b9"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E88113A-166D-44CD-886E-1102874B4258}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>